<commit_message>
Update ACT table through WK2639
</commit_message>
<xml_diff>
--- a/ACT table.xlsx
+++ b/ACT table.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\=Codex study==\20260604-Sites in Codex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D85FF412-C9E2-427F-B7CF-7918136D219F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F76A0EF-5F80-4E8B-A685-DEBE3D829114}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025 ACT" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="178">
   <si>
     <t>開賣年度</t>
   </si>
@@ -563,6 +563,12 @@
   <si>
     <t>W2637</t>
   </si>
+  <si>
+    <t>W2638</t>
+  </si>
+  <si>
+    <t>W2639</t>
+  </si>
 </sst>
 </file>
 
@@ -954,13 +960,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BU35"/>
-  <sheetFormatPr defaultRowHeight="16.75" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="25.23046875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="32.23046875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.25" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.25" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1181,7 +1187,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2025</v>
       </c>
@@ -1327,7 +1333,7 @@
         <v>32021</v>
       </c>
     </row>
-    <row r="3" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2025</v>
       </c>
@@ -1473,7 +1479,7 @@
         <v>24860</v>
       </c>
     </row>
-    <row r="4" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -1655,7 +1661,7 @@
         <v>258587</v>
       </c>
     </row>
-    <row r="5" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2025</v>
       </c>
@@ -1819,7 +1825,7 @@
         <v>605786</v>
       </c>
     </row>
-    <row r="6" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2025</v>
       </c>
@@ -1986,7 +1992,7 @@
         <v>178766</v>
       </c>
     </row>
-    <row r="7" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2025</v>
       </c>
@@ -2126,7 +2132,7 @@
         <v>34772</v>
       </c>
     </row>
-    <row r="8" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2025</v>
       </c>
@@ -2299,7 +2305,7 @@
         <v>69631</v>
       </c>
     </row>
-    <row r="9" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2025</v>
       </c>
@@ -2472,7 +2478,7 @@
         <v>81858</v>
       </c>
     </row>
-    <row r="10" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2025</v>
       </c>
@@ -2609,7 +2615,7 @@
         <v>48453</v>
       </c>
     </row>
-    <row r="11" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -2782,7 +2788,7 @@
         <v>109519</v>
       </c>
     </row>
-    <row r="12" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2025</v>
       </c>
@@ -2958,7 +2964,7 @@
         <v>18079</v>
       </c>
     </row>
-    <row r="13" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2025</v>
       </c>
@@ -3116,7 +3122,7 @@
         <v>18613</v>
       </c>
     </row>
-    <row r="14" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2025</v>
       </c>
@@ -3253,7 +3259,7 @@
         <v>12463</v>
       </c>
     </row>
-    <row r="15" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2025</v>
       </c>
@@ -3387,7 +3393,7 @@
         <v>8028</v>
       </c>
     </row>
-    <row r="16" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2025</v>
       </c>
@@ -3566,7 +3572,7 @@
         <v>98598</v>
       </c>
     </row>
-    <row r="17" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -3748,7 +3754,7 @@
         <v>41246</v>
       </c>
     </row>
-    <row r="18" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2025</v>
       </c>
@@ -3942,7 +3948,7 @@
         <v>34091</v>
       </c>
     </row>
-    <row r="19" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2025</v>
       </c>
@@ -4118,7 +4124,7 @@
         <v>20240</v>
       </c>
     </row>
-    <row r="20" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2025</v>
       </c>
@@ -4309,7 +4315,7 @@
         <v>21614</v>
       </c>
     </row>
-    <row r="21" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2025</v>
       </c>
@@ -4488,7 +4494,7 @@
         <v>49925</v>
       </c>
     </row>
-    <row r="22" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -4667,7 +4673,7 @@
         <v>48736</v>
       </c>
     </row>
-    <row r="23" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2025</v>
       </c>
@@ -4849,7 +4855,7 @@
         <v>52186</v>
       </c>
     </row>
-    <row r="24" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2025</v>
       </c>
@@ -4962,7 +4968,7 @@
         <v>12731</v>
       </c>
     </row>
-    <row r="25" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2025</v>
       </c>
@@ -5123,7 +5129,7 @@
         <v>39938</v>
       </c>
     </row>
-    <row r="26" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2025</v>
       </c>
@@ -5236,7 +5242,7 @@
         <v>18016</v>
       </c>
     </row>
-    <row r="27" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2025</v>
       </c>
@@ -5457,7 +5463,7 @@
         <v>58189</v>
       </c>
     </row>
-    <row r="28" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2025</v>
       </c>
@@ -5642,7 +5648,7 @@
         <v>24715</v>
       </c>
     </row>
-    <row r="29" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2025</v>
       </c>
@@ -5821,7 +5827,7 @@
         <v>5323</v>
       </c>
     </row>
-    <row r="30" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2025</v>
       </c>
@@ -6021,7 +6027,7 @@
         <v>105927</v>
       </c>
     </row>
-    <row r="31" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2025</v>
       </c>
@@ -6230,7 +6236,7 @@
         <v>11763</v>
       </c>
     </row>
-    <row r="32" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2025</v>
       </c>
@@ -6379,7 +6385,7 @@
         <v>15110</v>
       </c>
     </row>
-    <row r="33" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2025</v>
       </c>
@@ -6534,7 +6540,7 @@
         <v>23108</v>
       </c>
     </row>
-    <row r="34" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2025</v>
       </c>
@@ -6725,7 +6731,7 @@
         <v>46550</v>
       </c>
     </row>
-    <row r="35" spans="1:73" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:73" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2025</v>
       </c>
@@ -6919,15 +6925,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:GR49"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.75" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="25.23046875" customWidth="1"/>
-    <col min="3" max="3" width="32.23046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.25" customWidth="1"/>
+    <col min="3" max="3" width="32.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -7048,8 +7054,14 @@
       <c r="AN1" t="s">
         <v>175</v>
       </c>
+      <c r="AO1" t="s">
+        <v>176</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>177</v>
+      </c>
     </row>
-    <row r="2" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2026</v>
       </c>
@@ -7160,8 +7172,12 @@
       <c r="AN2" s="2">
         <v>5455</v>
       </c>
-      <c r="AO2" s="2"/>
-      <c r="AP2" s="2"/>
+      <c r="AO2" s="2">
+        <v>5720</v>
+      </c>
+      <c r="AP2" s="2">
+        <v>5985</v>
+      </c>
       <c r="AQ2" s="2"/>
       <c r="AR2" s="2"/>
       <c r="AS2" s="2"/>
@@ -7321,7 +7337,7 @@
       <c r="GQ2" s="2"/>
       <c r="GR2" s="2"/>
     </row>
-    <row r="3" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2026</v>
       </c>
@@ -7406,8 +7422,12 @@
       <c r="AN3" s="2">
         <v>0</v>
       </c>
-      <c r="AO3" s="2"/>
-      <c r="AP3" s="2"/>
+      <c r="AO3" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP3" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ3" s="2"/>
       <c r="AR3" s="2"/>
       <c r="AS3" s="2"/>
@@ -7567,7 +7587,7 @@
       <c r="GQ3" s="2"/>
       <c r="GR3" s="2"/>
     </row>
-    <row r="4" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2026</v>
       </c>
@@ -7672,8 +7692,12 @@
       <c r="AN4" s="2">
         <v>8302</v>
       </c>
-      <c r="AO4" s="2"/>
-      <c r="AP4" s="2"/>
+      <c r="AO4" s="2">
+        <v>8531</v>
+      </c>
+      <c r="AP4" s="2">
+        <v>8759</v>
+      </c>
       <c r="AQ4" s="2"/>
       <c r="AR4" s="2"/>
       <c r="AS4" s="2"/>
@@ -7833,7 +7857,7 @@
       <c r="GQ4" s="2"/>
       <c r="GR4" s="2"/>
     </row>
-    <row r="5" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2026</v>
       </c>
@@ -7926,8 +7950,12 @@
       <c r="AN5" s="2">
         <v>4366</v>
       </c>
-      <c r="AO5" s="2"/>
-      <c r="AP5" s="2"/>
+      <c r="AO5" s="2">
+        <v>4490</v>
+      </c>
+      <c r="AP5" s="2">
+        <v>4614</v>
+      </c>
       <c r="AQ5" s="2"/>
       <c r="AR5" s="2"/>
       <c r="AS5" s="2"/>
@@ -8087,7 +8115,7 @@
       <c r="GQ5" s="2"/>
       <c r="GR5" s="2"/>
     </row>
-    <row r="6" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -8154,8 +8182,12 @@
       <c r="AN6" s="2">
         <v>0</v>
       </c>
-      <c r="AO6" s="2"/>
-      <c r="AP6" s="2"/>
+      <c r="AO6" s="2">
+        <v>703</v>
+      </c>
+      <c r="AP6" s="2">
+        <v>1405</v>
+      </c>
       <c r="AQ6" s="2"/>
       <c r="AR6" s="2"/>
       <c r="AS6" s="2"/>
@@ -8315,7 +8347,7 @@
       <c r="GQ6" s="2"/>
       <c r="GR6" s="2"/>
     </row>
-    <row r="7" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -8400,8 +8432,12 @@
       <c r="AN7" s="2">
         <v>0</v>
       </c>
-      <c r="AO7" s="2"/>
-      <c r="AP7" s="2"/>
+      <c r="AO7" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP7" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ7" s="2"/>
       <c r="AR7" s="2"/>
       <c r="AS7" s="2"/>
@@ -8561,7 +8597,7 @@
       <c r="GQ7" s="2"/>
       <c r="GR7" s="2"/>
     </row>
-    <row r="8" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2026</v>
       </c>
@@ -8646,8 +8682,12 @@
       <c r="AN8" s="2">
         <v>0</v>
       </c>
-      <c r="AO8" s="2"/>
-      <c r="AP8" s="2"/>
+      <c r="AO8" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP8" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ8" s="2"/>
       <c r="AR8" s="2"/>
       <c r="AS8" s="2"/>
@@ -8807,7 +8847,7 @@
       <c r="GQ8" s="2"/>
       <c r="GR8" s="2"/>
     </row>
-    <row r="9" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2026</v>
       </c>
@@ -8892,8 +8932,12 @@
       <c r="AN9" s="2">
         <v>0</v>
       </c>
-      <c r="AO9" s="2"/>
-      <c r="AP9" s="2"/>
+      <c r="AO9" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP9" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ9" s="2"/>
       <c r="AR9" s="2"/>
       <c r="AS9" s="2"/>
@@ -9053,7 +9097,7 @@
       <c r="GQ9" s="2"/>
       <c r="GR9" s="2"/>
     </row>
-    <row r="10" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2026</v>
       </c>
@@ -9138,8 +9182,12 @@
       <c r="AN10" s="2">
         <v>0</v>
       </c>
-      <c r="AO10" s="2"/>
-      <c r="AP10" s="2"/>
+      <c r="AO10" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP10" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ10" s="2"/>
       <c r="AR10" s="2"/>
       <c r="AS10" s="2"/>
@@ -9299,7 +9347,7 @@
       <c r="GQ10" s="2"/>
       <c r="GR10" s="2"/>
     </row>
-    <row r="11" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2026</v>
       </c>
@@ -9384,8 +9432,12 @@
       <c r="AN11" s="2">
         <v>0</v>
       </c>
-      <c r="AO11" s="2"/>
-      <c r="AP11" s="2"/>
+      <c r="AO11" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP11" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ11" s="2"/>
       <c r="AR11" s="2"/>
       <c r="AS11" s="2"/>
@@ -9545,7 +9597,7 @@
       <c r="GQ11" s="2"/>
       <c r="GR11" s="2"/>
     </row>
-    <row r="12" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -9630,8 +9682,12 @@
       <c r="AN12" s="2">
         <v>15266</v>
       </c>
-      <c r="AO12" s="2"/>
-      <c r="AP12" s="2"/>
+      <c r="AO12" s="2">
+        <v>16292</v>
+      </c>
+      <c r="AP12" s="2">
+        <v>17317</v>
+      </c>
       <c r="AQ12" s="2"/>
       <c r="AR12" s="2"/>
       <c r="AS12" s="2"/>
@@ -9791,7 +9847,7 @@
       <c r="GQ12" s="2"/>
       <c r="GR12" s="2"/>
     </row>
-    <row r="13" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -9876,8 +9932,12 @@
       <c r="AN13" s="2">
         <v>133381</v>
       </c>
-      <c r="AO13" s="2"/>
-      <c r="AP13" s="2"/>
+      <c r="AO13" s="2">
+        <v>137564</v>
+      </c>
+      <c r="AP13" s="2">
+        <v>141747</v>
+      </c>
       <c r="AQ13" s="2"/>
       <c r="AR13" s="2"/>
       <c r="AS13" s="2"/>
@@ -10037,7 +10097,7 @@
       <c r="GQ13" s="2"/>
       <c r="GR13" s="2"/>
     </row>
-    <row r="14" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2026</v>
       </c>
@@ -10122,8 +10182,12 @@
       <c r="AN14" s="2">
         <v>22419</v>
       </c>
-      <c r="AO14" s="2"/>
-      <c r="AP14" s="2"/>
+      <c r="AO14" s="2">
+        <v>23002</v>
+      </c>
+      <c r="AP14" s="2">
+        <v>23585</v>
+      </c>
       <c r="AQ14" s="2"/>
       <c r="AR14" s="2"/>
       <c r="AS14" s="2"/>
@@ -10283,7 +10347,7 @@
       <c r="GQ14" s="2"/>
       <c r="GR14" s="2"/>
     </row>
-    <row r="15" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2026</v>
       </c>
@@ -10368,8 +10432,12 @@
       <c r="AN15" s="2">
         <v>845</v>
       </c>
-      <c r="AO15" s="2"/>
-      <c r="AP15" s="2"/>
+      <c r="AO15" s="2">
+        <v>945</v>
+      </c>
+      <c r="AP15" s="2">
+        <v>1044</v>
+      </c>
       <c r="AQ15" s="2"/>
       <c r="AR15" s="2"/>
       <c r="AS15" s="2"/>
@@ -10529,7 +10597,7 @@
       <c r="GQ15" s="2"/>
       <c r="GR15" s="2"/>
     </row>
-    <row r="16" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2026</v>
       </c>
@@ -10614,8 +10682,12 @@
       <c r="AN16" s="2">
         <v>1741</v>
       </c>
-      <c r="AO16" s="2"/>
-      <c r="AP16" s="2"/>
+      <c r="AO16" s="2">
+        <v>1880</v>
+      </c>
+      <c r="AP16" s="2">
+        <v>2019</v>
+      </c>
       <c r="AQ16" s="2"/>
       <c r="AR16" s="2"/>
       <c r="AS16" s="2"/>
@@ -10775,7 +10847,7 @@
       <c r="GQ16" s="2"/>
       <c r="GR16" s="2"/>
     </row>
-    <row r="17" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2026</v>
       </c>
@@ -10858,8 +10930,12 @@
       <c r="AN17" s="2">
         <v>1281</v>
       </c>
-      <c r="AO17" s="2"/>
-      <c r="AP17" s="2"/>
+      <c r="AO17" s="2">
+        <v>1345</v>
+      </c>
+      <c r="AP17" s="2">
+        <v>1408</v>
+      </c>
       <c r="AQ17" s="2"/>
       <c r="AR17" s="2"/>
       <c r="AS17" s="2"/>
@@ -11019,7 +11095,7 @@
       <c r="GQ17" s="2"/>
       <c r="GR17" s="2"/>
     </row>
-    <row r="18" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2026</v>
       </c>
@@ -11104,8 +11180,12 @@
       <c r="AN18" s="2">
         <v>1495</v>
       </c>
-      <c r="AO18" s="2"/>
-      <c r="AP18" s="2"/>
+      <c r="AO18" s="2">
+        <v>1574</v>
+      </c>
+      <c r="AP18" s="2">
+        <v>1653</v>
+      </c>
       <c r="AQ18" s="2"/>
       <c r="AR18" s="2"/>
       <c r="AS18" s="2"/>
@@ -11265,7 +11345,7 @@
       <c r="GQ18" s="2"/>
       <c r="GR18" s="2"/>
     </row>
-    <row r="19" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2026</v>
       </c>
@@ -11350,8 +11430,12 @@
       <c r="AN19" s="2">
         <v>0</v>
       </c>
-      <c r="AO19" s="2"/>
-      <c r="AP19" s="2"/>
+      <c r="AO19" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP19" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ19" s="2"/>
       <c r="AR19" s="2"/>
       <c r="AS19" s="2"/>
@@ -11511,7 +11595,7 @@
       <c r="GQ19" s="2"/>
       <c r="GR19" s="2"/>
     </row>
-    <row r="20" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2026</v>
       </c>
@@ -11596,8 +11680,12 @@
       <c r="AN20" s="2">
         <v>212</v>
       </c>
-      <c r="AO20" s="2"/>
-      <c r="AP20" s="2"/>
+      <c r="AO20" s="2">
+        <v>232</v>
+      </c>
+      <c r="AP20" s="2">
+        <v>252</v>
+      </c>
       <c r="AQ20" s="2"/>
       <c r="AR20" s="2"/>
       <c r="AS20" s="2"/>
@@ -11757,7 +11845,7 @@
       <c r="GQ20" s="2"/>
       <c r="GR20" s="2"/>
     </row>
-    <row r="21" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2026</v>
       </c>
@@ -11842,8 +11930,12 @@
       <c r="AN21" s="2">
         <v>0</v>
       </c>
-      <c r="AO21" s="2"/>
-      <c r="AP21" s="2"/>
+      <c r="AO21" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP21" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ21" s="2"/>
       <c r="AR21" s="2"/>
       <c r="AS21" s="2"/>
@@ -12003,7 +12095,7 @@
       <c r="GQ21" s="2"/>
       <c r="GR21" s="2"/>
     </row>
-    <row r="22" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2026</v>
       </c>
@@ -12088,8 +12180,12 @@
       <c r="AN22" s="2">
         <v>714</v>
       </c>
-      <c r="AO22" s="2"/>
-      <c r="AP22" s="2"/>
+      <c r="AO22" s="2">
+        <v>760</v>
+      </c>
+      <c r="AP22" s="2">
+        <v>805</v>
+      </c>
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
       <c r="AS22" s="2"/>
@@ -12249,7 +12345,7 @@
       <c r="GQ22" s="2"/>
       <c r="GR22" s="2"/>
     </row>
-    <row r="23" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2026</v>
       </c>
@@ -12334,8 +12430,12 @@
       <c r="AN23" s="2">
         <v>1223</v>
       </c>
-      <c r="AO23" s="2"/>
-      <c r="AP23" s="2"/>
+      <c r="AO23" s="2">
+        <v>1277</v>
+      </c>
+      <c r="AP23" s="2">
+        <v>1331</v>
+      </c>
       <c r="AQ23" s="2"/>
       <c r="AR23" s="2"/>
       <c r="AS23" s="2"/>
@@ -12495,7 +12595,7 @@
       <c r="GQ23" s="2"/>
       <c r="GR23" s="2"/>
     </row>
-    <row r="24" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2026</v>
       </c>
@@ -12580,8 +12680,12 @@
       <c r="AN24" s="2">
         <v>2701</v>
       </c>
-      <c r="AO24" s="2"/>
-      <c r="AP24" s="2"/>
+      <c r="AO24" s="2">
+        <v>2839</v>
+      </c>
+      <c r="AP24" s="2">
+        <v>2976</v>
+      </c>
       <c r="AQ24" s="2"/>
       <c r="AR24" s="2"/>
       <c r="AS24" s="2"/>
@@ -12741,7 +12845,7 @@
       <c r="GQ24" s="2"/>
       <c r="GR24" s="2"/>
     </row>
-    <row r="25" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2026</v>
       </c>
@@ -12826,8 +12930,12 @@
       <c r="AN25" s="2">
         <v>756</v>
       </c>
-      <c r="AO25" s="2"/>
-      <c r="AP25" s="2"/>
+      <c r="AO25" s="2">
+        <v>790</v>
+      </c>
+      <c r="AP25" s="2">
+        <v>823</v>
+      </c>
       <c r="AQ25" s="2"/>
       <c r="AR25" s="2"/>
       <c r="AS25" s="2"/>
@@ -12987,7 +13095,7 @@
       <c r="GQ25" s="2"/>
       <c r="GR25" s="2"/>
     </row>
-    <row r="26" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -13072,8 +13180,12 @@
       <c r="AN26" s="2">
         <v>1604</v>
       </c>
-      <c r="AO26" s="2"/>
-      <c r="AP26" s="2"/>
+      <c r="AO26" s="2">
+        <v>1741</v>
+      </c>
+      <c r="AP26" s="2">
+        <v>1877</v>
+      </c>
       <c r="AQ26" s="2"/>
       <c r="AR26" s="2"/>
       <c r="AS26" s="2"/>
@@ -13233,7 +13345,7 @@
       <c r="GQ26" s="2"/>
       <c r="GR26" s="2"/>
     </row>
-    <row r="27" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -13318,8 +13430,12 @@
       <c r="AN27" s="2">
         <v>2454</v>
       </c>
-      <c r="AO27" s="2"/>
-      <c r="AP27" s="2"/>
+      <c r="AO27" s="2">
+        <v>2650</v>
+      </c>
+      <c r="AP27" s="2">
+        <v>2846</v>
+      </c>
       <c r="AQ27" s="2"/>
       <c r="AR27" s="2"/>
       <c r="AS27" s="2"/>
@@ -13479,7 +13595,7 @@
       <c r="GQ27" s="2"/>
       <c r="GR27" s="2"/>
     </row>
-    <row r="28" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2026</v>
       </c>
@@ -13564,8 +13680,12 @@
       <c r="AN28" s="2">
         <v>896</v>
       </c>
-      <c r="AO28" s="2"/>
-      <c r="AP28" s="2"/>
+      <c r="AO28" s="2">
+        <v>943</v>
+      </c>
+      <c r="AP28" s="2">
+        <v>989</v>
+      </c>
       <c r="AQ28" s="2"/>
       <c r="AR28" s="2"/>
       <c r="AS28" s="2"/>
@@ -13725,7 +13845,7 @@
       <c r="GQ28" s="2"/>
       <c r="GR28" s="2"/>
     </row>
-    <row r="29" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2026</v>
       </c>
@@ -13810,8 +13930,12 @@
       <c r="AN29" s="2">
         <v>2051</v>
       </c>
-      <c r="AO29" s="2"/>
-      <c r="AP29" s="2"/>
+      <c r="AO29" s="2">
+        <v>2124</v>
+      </c>
+      <c r="AP29" s="2">
+        <v>2197</v>
+      </c>
       <c r="AQ29" s="2"/>
       <c r="AR29" s="2"/>
       <c r="AS29" s="2"/>
@@ -13971,7 +14095,7 @@
       <c r="GQ29" s="2"/>
       <c r="GR29" s="2"/>
     </row>
-    <row r="30" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2026</v>
       </c>
@@ -14068,8 +14192,12 @@
       <c r="AN30" s="2">
         <v>2685</v>
       </c>
-      <c r="AO30" s="2"/>
-      <c r="AP30" s="2"/>
+      <c r="AO30" s="2">
+        <v>2728</v>
+      </c>
+      <c r="AP30" s="2">
+        <v>2770</v>
+      </c>
       <c r="AQ30" s="2"/>
       <c r="AR30" s="2"/>
       <c r="AS30" s="2"/>
@@ -14229,7 +14357,7 @@
       <c r="GQ30" s="2"/>
       <c r="GR30" s="2"/>
     </row>
-    <row r="31" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2026</v>
       </c>
@@ -14314,8 +14442,12 @@
       <c r="AN31" s="2">
         <v>0</v>
       </c>
-      <c r="AO31" s="2"/>
-      <c r="AP31" s="2"/>
+      <c r="AO31" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP31" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ31" s="2"/>
       <c r="AR31" s="2"/>
       <c r="AS31" s="2"/>
@@ -14475,7 +14607,7 @@
       <c r="GQ31" s="2"/>
       <c r="GR31" s="2"/>
     </row>
-    <row r="32" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2026</v>
       </c>
@@ -14560,8 +14692,12 @@
       <c r="AN32" s="2">
         <v>0</v>
       </c>
-      <c r="AO32" s="2"/>
-      <c r="AP32" s="2"/>
+      <c r="AO32" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP32" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ32" s="2"/>
       <c r="AR32" s="2"/>
       <c r="AS32" s="2"/>
@@ -14721,7 +14857,7 @@
       <c r="GQ32" s="2"/>
       <c r="GR32" s="2"/>
     </row>
-    <row r="33" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2026</v>
       </c>
@@ -14806,8 +14942,12 @@
       <c r="AN33" s="2">
         <v>0</v>
       </c>
-      <c r="AO33" s="2"/>
-      <c r="AP33" s="2"/>
+      <c r="AO33" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP33" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ33" s="2"/>
       <c r="AR33" s="2"/>
       <c r="AS33" s="2"/>
@@ -14967,7 +15107,7 @@
       <c r="GQ33" s="2"/>
       <c r="GR33" s="2"/>
     </row>
-    <row r="34" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2026</v>
       </c>
@@ -15052,8 +15192,12 @@
       <c r="AN34" s="2">
         <v>0</v>
       </c>
-      <c r="AO34" s="2"/>
-      <c r="AP34" s="2"/>
+      <c r="AO34" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP34" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ34" s="2"/>
       <c r="AR34" s="2"/>
       <c r="AS34" s="2"/>
@@ -15213,7 +15357,7 @@
       <c r="GQ34" s="2"/>
       <c r="GR34" s="2"/>
     </row>
-    <row r="35" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2026</v>
       </c>
@@ -15324,8 +15468,12 @@
       <c r="AN35" s="2">
         <v>7601</v>
       </c>
-      <c r="AO35" s="2"/>
-      <c r="AP35" s="2"/>
+      <c r="AO35" s="2">
+        <v>7856</v>
+      </c>
+      <c r="AP35" s="2">
+        <v>8107</v>
+      </c>
       <c r="AQ35" s="2"/>
       <c r="AR35" s="2"/>
       <c r="AS35" s="2"/>
@@ -15485,7 +15633,7 @@
       <c r="GQ35" s="2"/>
       <c r="GR35" s="2"/>
     </row>
-    <row r="36" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2026</v>
       </c>
@@ -15570,8 +15718,12 @@
       <c r="AN36" s="2">
         <v>928</v>
       </c>
-      <c r="AO36" s="2"/>
-      <c r="AP36" s="2"/>
+      <c r="AO36" s="2">
+        <v>1001</v>
+      </c>
+      <c r="AP36" s="2">
+        <v>1050</v>
+      </c>
       <c r="AQ36" s="2"/>
       <c r="AR36" s="2"/>
       <c r="AS36" s="2"/>
@@ -15731,7 +15883,7 @@
       <c r="GQ36" s="2"/>
       <c r="GR36" s="2"/>
     </row>
-    <row r="37" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2026</v>
       </c>
@@ -15816,8 +15968,12 @@
       <c r="AN37" s="2">
         <v>1476</v>
       </c>
-      <c r="AO37" s="2"/>
-      <c r="AP37" s="2"/>
+      <c r="AO37" s="2">
+        <v>1649</v>
+      </c>
+      <c r="AP37" s="2">
+        <v>1771</v>
+      </c>
       <c r="AQ37" s="2"/>
       <c r="AR37" s="2"/>
       <c r="AS37" s="2"/>
@@ -15977,7 +16133,7 @@
       <c r="GQ37" s="2"/>
       <c r="GR37" s="2"/>
     </row>
-    <row r="38" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2026</v>
       </c>
@@ -16064,8 +16220,12 @@
       <c r="AN38" s="2">
         <v>4729</v>
       </c>
-      <c r="AO38" s="2"/>
-      <c r="AP38" s="2"/>
+      <c r="AO38" s="2">
+        <v>5217</v>
+      </c>
+      <c r="AP38" s="2">
+        <v>5652</v>
+      </c>
       <c r="AQ38" s="2"/>
       <c r="AR38" s="2"/>
       <c r="AS38" s="2"/>
@@ -16225,7 +16385,7 @@
       <c r="GQ38" s="2"/>
       <c r="GR38" s="2"/>
     </row>
-    <row r="39" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2026</v>
       </c>
@@ -16336,8 +16496,12 @@
       <c r="AN39" s="2">
         <v>10934</v>
       </c>
-      <c r="AO39" s="2"/>
-      <c r="AP39" s="2"/>
+      <c r="AO39" s="2">
+        <v>11499</v>
+      </c>
+      <c r="AP39" s="2">
+        <v>12143</v>
+      </c>
       <c r="AQ39" s="2"/>
       <c r="AR39" s="2"/>
       <c r="AS39" s="2"/>
@@ -16497,7 +16661,7 @@
       <c r="GQ39" s="2"/>
       <c r="GR39" s="2"/>
     </row>
-    <row r="40" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2026</v>
       </c>
@@ -16608,8 +16772,12 @@
       <c r="AN40" s="2">
         <v>4868</v>
       </c>
-      <c r="AO40" s="2"/>
-      <c r="AP40" s="2"/>
+      <c r="AO40" s="2">
+        <v>5263</v>
+      </c>
+      <c r="AP40" s="2">
+        <v>5581</v>
+      </c>
       <c r="AQ40" s="2"/>
       <c r="AR40" s="2"/>
       <c r="AS40" s="2"/>
@@ -16769,7 +16937,7 @@
       <c r="GQ40" s="2"/>
       <c r="GR40" s="2"/>
     </row>
-    <row r="41" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2026</v>
       </c>
@@ -16858,8 +17026,12 @@
       <c r="AN41" s="2">
         <v>9396</v>
       </c>
-      <c r="AO41" s="2"/>
-      <c r="AP41" s="2"/>
+      <c r="AO41" s="2">
+        <v>10043</v>
+      </c>
+      <c r="AP41" s="2">
+        <v>10620</v>
+      </c>
       <c r="AQ41" s="2"/>
       <c r="AR41" s="2"/>
       <c r="AS41" s="2"/>
@@ -17019,7 +17191,7 @@
       <c r="GQ41" s="2"/>
       <c r="GR41" s="2"/>
     </row>
-    <row r="42" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2026</v>
       </c>
@@ -17104,8 +17276,12 @@
       <c r="AN42" s="2">
         <v>0</v>
       </c>
-      <c r="AO42" s="2"/>
-      <c r="AP42" s="2"/>
+      <c r="AO42" s="2">
+        <v>433</v>
+      </c>
+      <c r="AP42" s="2">
+        <v>475</v>
+      </c>
       <c r="AQ42" s="2"/>
       <c r="AR42" s="2"/>
       <c r="AS42" s="2"/>
@@ -17265,7 +17441,7 @@
       <c r="GQ42" s="2"/>
       <c r="GR42" s="2"/>
     </row>
-    <row r="43" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2026</v>
       </c>
@@ -17350,8 +17526,12 @@
       <c r="AN43" s="2">
         <v>0</v>
       </c>
-      <c r="AO43" s="2"/>
-      <c r="AP43" s="2"/>
+      <c r="AO43" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP43" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ43" s="2"/>
       <c r="AR43" s="2"/>
       <c r="AS43" s="2"/>
@@ -17511,7 +17691,7 @@
       <c r="GQ43" s="2"/>
       <c r="GR43" s="2"/>
     </row>
-    <row r="44" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2026</v>
       </c>
@@ -17596,8 +17776,12 @@
       <c r="AN44" s="2">
         <v>0</v>
       </c>
-      <c r="AO44" s="2"/>
-      <c r="AP44" s="2"/>
+      <c r="AO44" s="2">
+        <v>0</v>
+      </c>
+      <c r="AP44" s="2">
+        <v>0</v>
+      </c>
       <c r="AQ44" s="2"/>
       <c r="AR44" s="2"/>
       <c r="AS44" s="2"/>
@@ -17757,7 +17941,7 @@
       <c r="GQ44" s="2"/>
       <c r="GR44" s="2"/>
     </row>
-    <row r="45" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2026</v>
       </c>
@@ -17868,8 +18052,12 @@
       <c r="AN45" s="2">
         <v>13941</v>
       </c>
-      <c r="AO45" s="2"/>
-      <c r="AP45" s="2"/>
+      <c r="AO45" s="2">
+        <v>14581</v>
+      </c>
+      <c r="AP45" s="2">
+        <v>15156</v>
+      </c>
       <c r="AQ45" s="2"/>
       <c r="AR45" s="2"/>
       <c r="AS45" s="2"/>
@@ -18029,7 +18217,7 @@
       <c r="GQ45" s="2"/>
       <c r="GR45" s="2"/>
     </row>
-    <row r="46" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2026</v>
       </c>
@@ -18114,8 +18302,12 @@
       <c r="AN46" s="2">
         <v>2306</v>
       </c>
-      <c r="AO46" s="2"/>
-      <c r="AP46" s="2"/>
+      <c r="AO46" s="2">
+        <v>2495</v>
+      </c>
+      <c r="AP46" s="2">
+        <v>2683</v>
+      </c>
       <c r="AQ46" s="2"/>
       <c r="AR46" s="2"/>
       <c r="AS46" s="2"/>
@@ -18275,7 +18467,7 @@
       <c r="GQ46" s="2"/>
       <c r="GR46" s="2"/>
     </row>
-    <row r="47" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2026</v>
       </c>
@@ -18360,8 +18552,12 @@
       <c r="AN47" s="2">
         <v>3809</v>
       </c>
-      <c r="AO47" s="2"/>
-      <c r="AP47" s="2"/>
+      <c r="AO47" s="2">
+        <v>3980</v>
+      </c>
+      <c r="AP47" s="2">
+        <v>4111</v>
+      </c>
       <c r="AQ47" s="2"/>
       <c r="AR47" s="2"/>
       <c r="AS47" s="2"/>
@@ -18521,7 +18717,7 @@
       <c r="GQ47" s="2"/>
       <c r="GR47" s="2"/>
     </row>
-    <row r="48" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2026</v>
       </c>
@@ -18606,8 +18802,12 @@
       <c r="AN48" s="2">
         <v>2726</v>
       </c>
-      <c r="AO48" s="2"/>
-      <c r="AP48" s="2"/>
+      <c r="AO48" s="2">
+        <v>3541</v>
+      </c>
+      <c r="AP48" s="2">
+        <v>4212</v>
+      </c>
       <c r="AQ48" s="2"/>
       <c r="AR48" s="2"/>
       <c r="AS48" s="2"/>
@@ -18767,7 +18967,7 @@
       <c r="GQ48" s="2"/>
       <c r="GR48" s="2"/>
     </row>
-    <row r="49" spans="1:200" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:200" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2026</v>
       </c>
@@ -18878,8 +19078,12 @@
       <c r="AN49" s="2">
         <v>10949</v>
       </c>
-      <c r="AO49" s="2"/>
-      <c r="AP49" s="2"/>
+      <c r="AO49" s="2">
+        <v>11500</v>
+      </c>
+      <c r="AP49" s="2">
+        <v>12172</v>
+      </c>
       <c r="AQ49" s="2"/>
       <c r="AR49" s="2"/>
       <c r="AS49" s="2"/>

</xml_diff>

<commit_message>
Persist W2641 ACT snapshot from verified uploaded workbook
</commit_message>
<xml_diff>
--- a/ACT table.xlsx
+++ b/ACT table.xlsx
@@ -6946,6 +6946,11 @@
           <t>W2640</t>
         </is>
       </c>
+      <c r="AR1" s="0" t="inlineStr">
+        <is>
+          <t>W2641</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -7071,7 +7076,9 @@
       <c r="AQ2" s="6" t="n">
         <v>6445</v>
       </c>
-      <c r="AR2" s="4" t="n"/>
+      <c r="AR2" s="6" t="n">
+        <v>7097</v>
+      </c>
       <c r="AS2" s="4" t="n"/>
       <c r="AT2" s="4" t="n"/>
       <c r="AU2" s="4" t="n"/>
@@ -7327,7 +7334,9 @@
       <c r="AQ3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR3" s="4" t="n"/>
+      <c r="AR3" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS3" s="4" t="n"/>
       <c r="AT3" s="4" t="n"/>
       <c r="AU3" s="4" t="n"/>
@@ -7603,7 +7612,9 @@
       <c r="AQ4" s="6" t="n">
         <v>8941</v>
       </c>
-      <c r="AR4" s="4" t="n"/>
+      <c r="AR4" s="6" t="n">
+        <v>9109</v>
+      </c>
       <c r="AS4" s="4" t="n"/>
       <c r="AT4" s="4" t="n"/>
       <c r="AU4" s="4" t="n"/>
@@ -7867,7 +7878,9 @@
       <c r="AQ5" s="6" t="n">
         <v>4744</v>
       </c>
-      <c r="AR5" s="4" t="n"/>
+      <c r="AR5" s="6" t="n">
+        <v>4788</v>
+      </c>
       <c r="AS5" s="4" t="n"/>
       <c r="AT5" s="4" t="n"/>
       <c r="AU5" s="4" t="n"/>
@@ -8105,7 +8118,9 @@
       <c r="AQ6" s="6" t="n">
         <v>1405</v>
       </c>
-      <c r="AR6" s="4" t="n"/>
+      <c r="AR6" s="6" t="n">
+        <v>2736</v>
+      </c>
       <c r="AS6" s="4" t="n"/>
       <c r="AT6" s="4" t="n"/>
       <c r="AU6" s="4" t="n"/>
@@ -8361,7 +8376,9 @@
       <c r="AQ7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR7" s="4" t="n"/>
+      <c r="AR7" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS7" s="4" t="n"/>
       <c r="AT7" s="4" t="n"/>
       <c r="AU7" s="4" t="n"/>
@@ -8617,7 +8634,9 @@
       <c r="AQ8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR8" s="4" t="n"/>
+      <c r="AR8" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS8" s="4" t="n"/>
       <c r="AT8" s="4" t="n"/>
       <c r="AU8" s="4" t="n"/>
@@ -8873,7 +8892,9 @@
       <c r="AQ9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR9" s="4" t="n"/>
+      <c r="AR9" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS9" s="4" t="n"/>
       <c r="AT9" s="4" t="n"/>
       <c r="AU9" s="4" t="n"/>
@@ -9129,7 +9150,9 @@
       <c r="AQ10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR10" s="4" t="n"/>
+      <c r="AR10" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS10" s="4" t="n"/>
       <c r="AT10" s="4" t="n"/>
       <c r="AU10" s="4" t="n"/>
@@ -9385,7 +9408,9 @@
       <c r="AQ11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR11" s="4" t="n"/>
+      <c r="AR11" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS11" s="4" t="n"/>
       <c r="AT11" s="4" t="n"/>
       <c r="AU11" s="4" t="n"/>
@@ -9641,7 +9666,9 @@
       <c r="AQ12" s="6" t="n">
         <v>19502</v>
       </c>
-      <c r="AR12" s="4" t="n"/>
+      <c r="AR12" s="6" t="n">
+        <v>21013</v>
+      </c>
       <c r="AS12" s="4" t="n"/>
       <c r="AT12" s="4" t="n"/>
       <c r="AU12" s="4" t="n"/>
@@ -9897,7 +9924,9 @@
       <c r="AQ13" s="6" t="n">
         <v>152638</v>
       </c>
-      <c r="AR13" s="4" t="n"/>
+      <c r="AR13" s="6" t="n">
+        <v>159195</v>
+      </c>
       <c r="AS13" s="4" t="n"/>
       <c r="AT13" s="4" t="n"/>
       <c r="AU13" s="4" t="n"/>
@@ -10153,7 +10182,9 @@
       <c r="AQ14" s="6" t="n">
         <v>24833</v>
       </c>
-      <c r="AR14" s="4" t="n"/>
+      <c r="AR14" s="6" t="n">
+        <v>25637</v>
+      </c>
       <c r="AS14" s="4" t="n"/>
       <c r="AT14" s="4" t="n"/>
       <c r="AU14" s="4" t="n"/>
@@ -10409,7 +10440,9 @@
       <c r="AQ15" s="6" t="n">
         <v>1156</v>
       </c>
-      <c r="AR15" s="4" t="n"/>
+      <c r="AR15" s="6" t="n">
+        <v>1156</v>
+      </c>
       <c r="AS15" s="4" t="n"/>
       <c r="AT15" s="4" t="n"/>
       <c r="AU15" s="4" t="n"/>
@@ -10665,7 +10698,9 @@
       <c r="AQ16" s="6" t="n">
         <v>2214</v>
       </c>
-      <c r="AR16" s="4" t="n"/>
+      <c r="AR16" s="6" t="n">
+        <v>2214</v>
+      </c>
       <c r="AS16" s="4" t="n"/>
       <c r="AT16" s="4" t="n"/>
       <c r="AU16" s="4" t="n"/>
@@ -10919,7 +10954,9 @@
       <c r="AQ17" s="6" t="n">
         <v>1560</v>
       </c>
-      <c r="AR17" s="4" t="n"/>
+      <c r="AR17" s="6" t="n">
+        <v>1643</v>
+      </c>
       <c r="AS17" s="4" t="n"/>
       <c r="AT17" s="4" t="n"/>
       <c r="AU17" s="4" t="n"/>
@@ -11175,7 +11212,9 @@
       <c r="AQ18" s="6" t="n">
         <v>1751</v>
       </c>
-      <c r="AR18" s="4" t="n"/>
+      <c r="AR18" s="6" t="n">
+        <v>1836</v>
+      </c>
       <c r="AS18" s="4" t="n"/>
       <c r="AT18" s="4" t="n"/>
       <c r="AU18" s="4" t="n"/>
@@ -11431,7 +11470,9 @@
       <c r="AQ19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR19" s="4" t="n"/>
+      <c r="AR19" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS19" s="4" t="n"/>
       <c r="AT19" s="4" t="n"/>
       <c r="AU19" s="4" t="n"/>
@@ -11687,7 +11728,9 @@
       <c r="AQ20" s="6" t="n">
         <v>252</v>
       </c>
-      <c r="AR20" s="4" t="n"/>
+      <c r="AR20" s="6" t="n">
+        <v>252</v>
+      </c>
       <c r="AS20" s="4" t="n"/>
       <c r="AT20" s="4" t="n"/>
       <c r="AU20" s="4" t="n"/>
@@ -11943,7 +11986,9 @@
       <c r="AQ21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR21" s="4" t="n"/>
+      <c r="AR21" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS21" s="4" t="n"/>
       <c r="AT21" s="4" t="n"/>
       <c r="AU21" s="4" t="n"/>
@@ -12199,7 +12244,9 @@
       <c r="AQ22" s="6" t="n">
         <v>805</v>
       </c>
-      <c r="AR22" s="4" t="n"/>
+      <c r="AR22" s="6" t="n">
+        <v>920</v>
+      </c>
       <c r="AS22" s="4" t="n"/>
       <c r="AT22" s="4" t="n"/>
       <c r="AU22" s="4" t="n"/>
@@ -12455,7 +12502,9 @@
       <c r="AQ23" s="6" t="n">
         <v>1331</v>
       </c>
-      <c r="AR23" s="4" t="n"/>
+      <c r="AR23" s="6" t="n">
+        <v>1480</v>
+      </c>
       <c r="AS23" s="4" t="n"/>
       <c r="AT23" s="4" t="n"/>
       <c r="AU23" s="4" t="n"/>
@@ -12711,7 +12760,9 @@
       <c r="AQ24" s="6" t="n">
         <v>3127</v>
       </c>
-      <c r="AR24" s="4" t="n"/>
+      <c r="AR24" s="6" t="n">
+        <v>3246</v>
+      </c>
       <c r="AS24" s="4" t="n"/>
       <c r="AT24" s="4" t="n"/>
       <c r="AU24" s="4" t="n"/>
@@ -12967,7 +13018,9 @@
       <c r="AQ25" s="6" t="n">
         <v>853</v>
       </c>
-      <c r="AR25" s="4" t="n"/>
+      <c r="AR25" s="6" t="n">
+        <v>877</v>
+      </c>
       <c r="AS25" s="4" t="n"/>
       <c r="AT25" s="4" t="n"/>
       <c r="AU25" s="4" t="n"/>
@@ -13223,7 +13276,9 @@
       <c r="AQ26" s="6" t="n">
         <v>2061</v>
       </c>
-      <c r="AR26" s="4" t="n"/>
+      <c r="AR26" s="6" t="n">
+        <v>2185</v>
+      </c>
       <c r="AS26" s="4" t="n"/>
       <c r="AT26" s="4" t="n"/>
       <c r="AU26" s="4" t="n"/>
@@ -13479,7 +13534,9 @@
       <c r="AQ27" s="6" t="n">
         <v>3049</v>
       </c>
-      <c r="AR27" s="4" t="n"/>
+      <c r="AR27" s="6" t="n">
+        <v>3049</v>
+      </c>
       <c r="AS27" s="4" t="n"/>
       <c r="AT27" s="4" t="n"/>
       <c r="AU27" s="4" t="n"/>
@@ -13735,7 +13792,9 @@
       <c r="AQ28" s="6" t="n">
         <v>1036</v>
       </c>
-      <c r="AR28" s="4" t="n"/>
+      <c r="AR28" s="6" t="n">
+        <v>1080</v>
+      </c>
       <c r="AS28" s="4" t="n"/>
       <c r="AT28" s="4" t="n"/>
       <c r="AU28" s="4" t="n"/>
@@ -13991,7 +14050,9 @@
       <c r="AQ29" s="6" t="n">
         <v>2276</v>
       </c>
-      <c r="AR29" s="4" t="n"/>
+      <c r="AR29" s="6" t="n">
+        <v>2351</v>
+      </c>
       <c r="AS29" s="4" t="n"/>
       <c r="AT29" s="4" t="n"/>
       <c r="AU29" s="4" t="n"/>
@@ -14259,7 +14320,9 @@
       <c r="AQ30" s="6" t="n">
         <v>2803</v>
       </c>
-      <c r="AR30" s="4" t="n"/>
+      <c r="AR30" s="6" t="n">
+        <v>2837</v>
+      </c>
       <c r="AS30" s="4" t="n"/>
       <c r="AT30" s="4" t="n"/>
       <c r="AU30" s="4" t="n"/>
@@ -14515,7 +14578,9 @@
       <c r="AQ31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR31" s="4" t="n"/>
+      <c r="AR31" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS31" s="4" t="n"/>
       <c r="AT31" s="4" t="n"/>
       <c r="AU31" s="4" t="n"/>
@@ -14771,7 +14836,9 @@
       <c r="AQ32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR32" s="4" t="n"/>
+      <c r="AR32" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS32" s="4" t="n"/>
       <c r="AT32" s="4" t="n"/>
       <c r="AU32" s="4" t="n"/>
@@ -15027,7 +15094,9 @@
       <c r="AQ33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR33" s="4" t="n"/>
+      <c r="AR33" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS33" s="4" t="n"/>
       <c r="AT33" s="4" t="n"/>
       <c r="AU33" s="4" t="n"/>
@@ -15283,7 +15352,9 @@
       <c r="AQ34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR34" s="4" t="n"/>
+      <c r="AR34" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS34" s="4" t="n"/>
       <c r="AT34" s="4" t="n"/>
       <c r="AU34" s="4" t="n"/>
@@ -15565,7 +15636,9 @@
       <c r="AQ35" s="6" t="n">
         <v>8360</v>
       </c>
-      <c r="AR35" s="4" t="n"/>
+      <c r="AR35" s="6" t="n">
+        <v>8618</v>
+      </c>
       <c r="AS35" s="4" t="n"/>
       <c r="AT35" s="4" t="n"/>
       <c r="AU35" s="4" t="n"/>
@@ -15821,7 +15894,9 @@
       <c r="AQ36" s="6" t="n">
         <v>1103</v>
       </c>
-      <c r="AR36" s="4" t="n"/>
+      <c r="AR36" s="6" t="n">
+        <v>1103</v>
+      </c>
       <c r="AS36" s="4" t="n"/>
       <c r="AT36" s="4" t="n"/>
       <c r="AU36" s="4" t="n"/>
@@ -16077,7 +16152,9 @@
       <c r="AQ37" s="6" t="n">
         <v>1859</v>
       </c>
-      <c r="AR37" s="4" t="n"/>
+      <c r="AR37" s="6" t="n">
+        <v>1962</v>
+      </c>
       <c r="AS37" s="4" t="n"/>
       <c r="AT37" s="4" t="n"/>
       <c r="AU37" s="4" t="n"/>
@@ -16335,7 +16412,9 @@
       <c r="AQ38" s="6" t="n">
         <v>6028</v>
       </c>
-      <c r="AR38" s="4" t="n"/>
+      <c r="AR38" s="6" t="n">
+        <v>6416</v>
+      </c>
       <c r="AS38" s="4" t="n"/>
       <c r="AT38" s="4" t="n"/>
       <c r="AU38" s="4" t="n"/>
@@ -16617,7 +16696,9 @@
       <c r="AQ39" s="6" t="n">
         <v>12831</v>
       </c>
-      <c r="AR39" s="4" t="n"/>
+      <c r="AR39" s="6" t="n">
+        <v>13529</v>
+      </c>
       <c r="AS39" s="4" t="n"/>
       <c r="AT39" s="4" t="n"/>
       <c r="AU39" s="4" t="n"/>
@@ -16899,7 +16980,9 @@
       <c r="AQ40" s="6" t="n">
         <v>5810</v>
       </c>
-      <c r="AR40" s="4" t="n"/>
+      <c r="AR40" s="6" t="n">
+        <v>6091</v>
+      </c>
       <c r="AS40" s="4" t="n"/>
       <c r="AT40" s="4" t="n"/>
       <c r="AU40" s="4" t="n"/>
@@ -17159,7 +17242,9 @@
       <c r="AQ41" s="6" t="n">
         <v>11338</v>
       </c>
-      <c r="AR41" s="4" t="n"/>
+      <c r="AR41" s="6" t="n">
+        <v>12178</v>
+      </c>
       <c r="AS41" s="4" t="n"/>
       <c r="AT41" s="4" t="n"/>
       <c r="AU41" s="4" t="n"/>
@@ -17415,7 +17500,9 @@
       <c r="AQ42" s="6" t="n">
         <v>475</v>
       </c>
-      <c r="AR42" s="4" t="n"/>
+      <c r="AR42" s="6" t="n">
+        <v>475</v>
+      </c>
       <c r="AS42" s="4" t="n"/>
       <c r="AT42" s="4" t="n"/>
       <c r="AU42" s="4" t="n"/>
@@ -17671,7 +17758,9 @@
       <c r="AQ43" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR43" s="4" t="n"/>
+      <c r="AR43" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS43" s="4" t="n"/>
       <c r="AT43" s="4" t="n"/>
       <c r="AU43" s="4" t="n"/>
@@ -17927,7 +18016,9 @@
       <c r="AQ44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AR44" s="4" t="n"/>
+      <c r="AR44" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AS44" s="4" t="n"/>
       <c r="AT44" s="4" t="n"/>
       <c r="AU44" s="4" t="n"/>
@@ -18209,7 +18300,9 @@
       <c r="AQ45" s="6" t="n">
         <v>15688</v>
       </c>
-      <c r="AR45" s="4" t="n"/>
+      <c r="AR45" s="6" t="n">
+        <v>16298</v>
+      </c>
       <c r="AS45" s="4" t="n"/>
       <c r="AT45" s="4" t="n"/>
       <c r="AU45" s="4" t="n"/>
@@ -18465,7 +18558,9 @@
       <c r="AQ46" s="6" t="n">
         <v>2864</v>
       </c>
-      <c r="AR46" s="4" t="n"/>
+      <c r="AR46" s="6" t="n">
+        <v>3081</v>
+      </c>
       <c r="AS46" s="4" t="n"/>
       <c r="AT46" s="4" t="n"/>
       <c r="AU46" s="4" t="n"/>
@@ -18721,7 +18816,9 @@
       <c r="AQ47" s="6" t="n">
         <v>4270</v>
       </c>
-      <c r="AR47" s="4" t="n"/>
+      <c r="AR47" s="6" t="n">
+        <v>4390</v>
+      </c>
       <c r="AS47" s="4" t="n"/>
       <c r="AT47" s="4" t="n"/>
       <c r="AU47" s="4" t="n"/>
@@ -18977,7 +19074,9 @@
       <c r="AQ48" s="6" t="n">
         <v>4710</v>
       </c>
-      <c r="AR48" s="4" t="n"/>
+      <c r="AR48" s="6" t="n">
+        <v>4710</v>
+      </c>
       <c r="AS48" s="4" t="n"/>
       <c r="AT48" s="4" t="n"/>
       <c r="AU48" s="4" t="n"/>
@@ -19259,7 +19358,9 @@
       <c r="AQ49" s="6" t="n">
         <v>12894</v>
       </c>
-      <c r="AR49" s="4" t="n"/>
+      <c r="AR49" s="6" t="n">
+        <v>13460</v>
+      </c>
       <c r="AS49" s="4" t="n"/>
       <c r="AT49" s="4" t="n"/>
       <c r="AU49" s="4" t="n"/>

</xml_diff>

<commit_message>
Update W2642 ACT snapshot (automatic)
</commit_message>
<xml_diff>
--- a/ACT table.xlsx
+++ b/ACT table.xlsx
@@ -6951,6 +6951,11 @@
           <t>W2641</t>
         </is>
       </c>
+      <c r="AS1" s="0" t="inlineStr">
+        <is>
+          <t>W2642</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -7079,7 +7084,9 @@
       <c r="AR2" s="6" t="n">
         <v>7097</v>
       </c>
-      <c r="AS2" s="4" t="n"/>
+      <c r="AS2" s="6" t="n">
+        <v>7626</v>
+      </c>
       <c r="AT2" s="4" t="n"/>
       <c r="AU2" s="4" t="n"/>
       <c r="AV2" s="4" t="n"/>
@@ -7337,7 +7344,9 @@
       <c r="AR3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS3" s="4" t="n"/>
+      <c r="AS3" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT3" s="4" t="n"/>
       <c r="AU3" s="4" t="n"/>
       <c r="AV3" s="4" t="n"/>
@@ -7615,7 +7624,9 @@
       <c r="AR4" s="6" t="n">
         <v>9109</v>
       </c>
-      <c r="AS4" s="4" t="n"/>
+      <c r="AS4" s="6" t="n">
+        <v>9261</v>
+      </c>
       <c r="AT4" s="4" t="n"/>
       <c r="AU4" s="4" t="n"/>
       <c r="AV4" s="4" t="n"/>
@@ -7881,7 +7892,9 @@
       <c r="AR5" s="6" t="n">
         <v>4788</v>
       </c>
-      <c r="AS5" s="4" t="n"/>
+      <c r="AS5" s="6" t="n">
+        <v>4835</v>
+      </c>
       <c r="AT5" s="4" t="n"/>
       <c r="AU5" s="4" t="n"/>
       <c r="AV5" s="4" t="n"/>
@@ -8121,7 +8134,9 @@
       <c r="AR6" s="6" t="n">
         <v>2736</v>
       </c>
-      <c r="AS6" s="4" t="n"/>
+      <c r="AS6" s="6" t="n">
+        <v>3913</v>
+      </c>
       <c r="AT6" s="4" t="n"/>
       <c r="AU6" s="4" t="n"/>
       <c r="AV6" s="4" t="n"/>
@@ -8379,7 +8394,9 @@
       <c r="AR7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS7" s="4" t="n"/>
+      <c r="AS7" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT7" s="4" t="n"/>
       <c r="AU7" s="4" t="n"/>
       <c r="AV7" s="4" t="n"/>
@@ -8637,7 +8654,9 @@
       <c r="AR8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS8" s="4" t="n"/>
+      <c r="AS8" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT8" s="4" t="n"/>
       <c r="AU8" s="4" t="n"/>
       <c r="AV8" s="4" t="n"/>
@@ -8895,7 +8914,9 @@
       <c r="AR9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS9" s="4" t="n"/>
+      <c r="AS9" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT9" s="4" t="n"/>
       <c r="AU9" s="4" t="n"/>
       <c r="AV9" s="4" t="n"/>
@@ -9153,7 +9174,9 @@
       <c r="AR10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS10" s="4" t="n"/>
+      <c r="AS10" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT10" s="4" t="n"/>
       <c r="AU10" s="4" t="n"/>
       <c r="AV10" s="4" t="n"/>
@@ -9411,7 +9434,9 @@
       <c r="AR11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS11" s="4" t="n"/>
+      <c r="AS11" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT11" s="4" t="n"/>
       <c r="AU11" s="4" t="n"/>
       <c r="AV11" s="4" t="n"/>
@@ -9669,7 +9694,9 @@
       <c r="AR12" s="6" t="n">
         <v>21013</v>
       </c>
-      <c r="AS12" s="4" t="n"/>
+      <c r="AS12" s="6" t="n">
+        <v>21823</v>
+      </c>
       <c r="AT12" s="4" t="n"/>
       <c r="AU12" s="4" t="n"/>
       <c r="AV12" s="4" t="n"/>
@@ -9927,7 +9954,9 @@
       <c r="AR13" s="6" t="n">
         <v>159195</v>
       </c>
-      <c r="AS13" s="4" t="n"/>
+      <c r="AS13" s="6" t="n">
+        <v>162837</v>
+      </c>
       <c r="AT13" s="4" t="n"/>
       <c r="AU13" s="4" t="n"/>
       <c r="AV13" s="4" t="n"/>
@@ -10185,7 +10214,9 @@
       <c r="AR14" s="6" t="n">
         <v>25637</v>
       </c>
-      <c r="AS14" s="4" t="n"/>
+      <c r="AS14" s="6" t="n">
+        <v>26198</v>
+      </c>
       <c r="AT14" s="4" t="n"/>
       <c r="AU14" s="4" t="n"/>
       <c r="AV14" s="4" t="n"/>
@@ -10443,7 +10474,9 @@
       <c r="AR15" s="6" t="n">
         <v>1156</v>
       </c>
-      <c r="AS15" s="4" t="n"/>
+      <c r="AS15" s="6" t="n">
+        <v>1156</v>
+      </c>
       <c r="AT15" s="4" t="n"/>
       <c r="AU15" s="4" t="n"/>
       <c r="AV15" s="4" t="n"/>
@@ -10701,7 +10734,9 @@
       <c r="AR16" s="6" t="n">
         <v>2214</v>
       </c>
-      <c r="AS16" s="4" t="n"/>
+      <c r="AS16" s="6" t="n">
+        <v>2491</v>
+      </c>
       <c r="AT16" s="4" t="n"/>
       <c r="AU16" s="4" t="n"/>
       <c r="AV16" s="4" t="n"/>
@@ -10957,7 +10992,9 @@
       <c r="AR17" s="6" t="n">
         <v>1643</v>
       </c>
-      <c r="AS17" s="4" t="n"/>
+      <c r="AS17" s="6" t="n">
+        <v>1717</v>
+      </c>
       <c r="AT17" s="4" t="n"/>
       <c r="AU17" s="4" t="n"/>
       <c r="AV17" s="4" t="n"/>
@@ -11215,7 +11252,9 @@
       <c r="AR18" s="6" t="n">
         <v>1836</v>
       </c>
-      <c r="AS18" s="4" t="n"/>
+      <c r="AS18" s="6" t="n">
+        <v>1922</v>
+      </c>
       <c r="AT18" s="4" t="n"/>
       <c r="AU18" s="4" t="n"/>
       <c r="AV18" s="4" t="n"/>
@@ -11473,7 +11512,9 @@
       <c r="AR19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS19" s="4" t="n"/>
+      <c r="AS19" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT19" s="4" t="n"/>
       <c r="AU19" s="4" t="n"/>
       <c r="AV19" s="4" t="n"/>
@@ -11731,7 +11772,9 @@
       <c r="AR20" s="6" t="n">
         <v>252</v>
       </c>
-      <c r="AS20" s="4" t="n"/>
+      <c r="AS20" s="6" t="n">
+        <v>252</v>
+      </c>
       <c r="AT20" s="4" t="n"/>
       <c r="AU20" s="4" t="n"/>
       <c r="AV20" s="4" t="n"/>
@@ -11989,7 +12032,9 @@
       <c r="AR21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS21" s="4" t="n"/>
+      <c r="AS21" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT21" s="4" t="n"/>
       <c r="AU21" s="4" t="n"/>
       <c r="AV21" s="4" t="n"/>
@@ -12247,7 +12292,9 @@
       <c r="AR22" s="6" t="n">
         <v>920</v>
       </c>
-      <c r="AS22" s="4" t="n"/>
+      <c r="AS22" s="6" t="n">
+        <v>956</v>
+      </c>
       <c r="AT22" s="4" t="n"/>
       <c r="AU22" s="4" t="n"/>
       <c r="AV22" s="4" t="n"/>
@@ -12505,7 +12552,9 @@
       <c r="AR23" s="6" t="n">
         <v>1480</v>
       </c>
-      <c r="AS23" s="4" t="n"/>
+      <c r="AS23" s="6" t="n">
+        <v>1515</v>
+      </c>
       <c r="AT23" s="4" t="n"/>
       <c r="AU23" s="4" t="n"/>
       <c r="AV23" s="4" t="n"/>
@@ -12763,7 +12812,9 @@
       <c r="AR24" s="6" t="n">
         <v>3246</v>
       </c>
-      <c r="AS24" s="4" t="n"/>
+      <c r="AS24" s="6" t="n">
+        <v>3363</v>
+      </c>
       <c r="AT24" s="4" t="n"/>
       <c r="AU24" s="4" t="n"/>
       <c r="AV24" s="4" t="n"/>
@@ -13021,7 +13072,9 @@
       <c r="AR25" s="6" t="n">
         <v>877</v>
       </c>
-      <c r="AS25" s="4" t="n"/>
+      <c r="AS25" s="6" t="n">
+        <v>877</v>
+      </c>
       <c r="AT25" s="4" t="n"/>
       <c r="AU25" s="4" t="n"/>
       <c r="AV25" s="4" t="n"/>
@@ -13279,7 +13332,9 @@
       <c r="AR26" s="6" t="n">
         <v>2185</v>
       </c>
-      <c r="AS26" s="4" t="n"/>
+      <c r="AS26" s="6" t="n">
+        <v>2300</v>
+      </c>
       <c r="AT26" s="4" t="n"/>
       <c r="AU26" s="4" t="n"/>
       <c r="AV26" s="4" t="n"/>
@@ -13537,7 +13592,9 @@
       <c r="AR27" s="6" t="n">
         <v>3049</v>
       </c>
-      <c r="AS27" s="4" t="n"/>
+      <c r="AS27" s="6" t="n">
+        <v>3458</v>
+      </c>
       <c r="AT27" s="4" t="n"/>
       <c r="AU27" s="4" t="n"/>
       <c r="AV27" s="4" t="n"/>
@@ -13795,7 +13852,9 @@
       <c r="AR28" s="6" t="n">
         <v>1080</v>
       </c>
-      <c r="AS28" s="4" t="n"/>
+      <c r="AS28" s="6" t="n">
+        <v>1113</v>
+      </c>
       <c r="AT28" s="4" t="n"/>
       <c r="AU28" s="4" t="n"/>
       <c r="AV28" s="4" t="n"/>
@@ -14053,7 +14112,9 @@
       <c r="AR29" s="6" t="n">
         <v>2351</v>
       </c>
-      <c r="AS29" s="4" t="n"/>
+      <c r="AS29" s="6" t="n">
+        <v>2417</v>
+      </c>
       <c r="AT29" s="4" t="n"/>
       <c r="AU29" s="4" t="n"/>
       <c r="AV29" s="4" t="n"/>
@@ -14323,7 +14384,9 @@
       <c r="AR30" s="6" t="n">
         <v>2837</v>
       </c>
-      <c r="AS30" s="4" t="n"/>
+      <c r="AS30" s="6" t="n">
+        <v>2868</v>
+      </c>
       <c r="AT30" s="4" t="n"/>
       <c r="AU30" s="4" t="n"/>
       <c r="AV30" s="4" t="n"/>
@@ -14581,7 +14644,9 @@
       <c r="AR31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS31" s="4" t="n"/>
+      <c r="AS31" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT31" s="4" t="n"/>
       <c r="AU31" s="4" t="n"/>
       <c r="AV31" s="4" t="n"/>
@@ -14839,7 +14904,9 @@
       <c r="AR32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS32" s="4" t="n"/>
+      <c r="AS32" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT32" s="4" t="n"/>
       <c r="AU32" s="4" t="n"/>
       <c r="AV32" s="4" t="n"/>
@@ -15097,7 +15164,9 @@
       <c r="AR33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS33" s="4" t="n"/>
+      <c r="AS33" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT33" s="4" t="n"/>
       <c r="AU33" s="4" t="n"/>
       <c r="AV33" s="4" t="n"/>
@@ -15355,7 +15424,9 @@
       <c r="AR34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS34" s="4" t="n"/>
+      <c r="AS34" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT34" s="4" t="n"/>
       <c r="AU34" s="4" t="n"/>
       <c r="AV34" s="4" t="n"/>
@@ -15639,7 +15710,9 @@
       <c r="AR35" s="6" t="n">
         <v>8618</v>
       </c>
-      <c r="AS35" s="4" t="n"/>
+      <c r="AS35" s="6" t="n">
+        <v>8823</v>
+      </c>
       <c r="AT35" s="4" t="n"/>
       <c r="AU35" s="4" t="n"/>
       <c r="AV35" s="4" t="n"/>
@@ -15897,7 +15970,9 @@
       <c r="AR36" s="6" t="n">
         <v>1103</v>
       </c>
-      <c r="AS36" s="4" t="n"/>
+      <c r="AS36" s="6" t="n">
+        <v>1189</v>
+      </c>
       <c r="AT36" s="4" t="n"/>
       <c r="AU36" s="4" t="n"/>
       <c r="AV36" s="4" t="n"/>
@@ -16155,7 +16230,9 @@
       <c r="AR37" s="6" t="n">
         <v>1962</v>
       </c>
-      <c r="AS37" s="4" t="n"/>
+      <c r="AS37" s="6" t="n">
+        <v>1962</v>
+      </c>
       <c r="AT37" s="4" t="n"/>
       <c r="AU37" s="4" t="n"/>
       <c r="AV37" s="4" t="n"/>
@@ -16415,7 +16492,9 @@
       <c r="AR38" s="6" t="n">
         <v>6416</v>
       </c>
-      <c r="AS38" s="4" t="n"/>
+      <c r="AS38" s="6" t="n">
+        <v>6853</v>
+      </c>
       <c r="AT38" s="4" t="n"/>
       <c r="AU38" s="4" t="n"/>
       <c r="AV38" s="4" t="n"/>
@@ -16699,7 +16778,9 @@
       <c r="AR39" s="6" t="n">
         <v>13529</v>
       </c>
-      <c r="AS39" s="4" t="n"/>
+      <c r="AS39" s="6" t="n">
+        <v>14183</v>
+      </c>
       <c r="AT39" s="4" t="n"/>
       <c r="AU39" s="4" t="n"/>
       <c r="AV39" s="4" t="n"/>
@@ -16983,7 +17064,9 @@
       <c r="AR40" s="6" t="n">
         <v>6091</v>
       </c>
-      <c r="AS40" s="4" t="n"/>
+      <c r="AS40" s="6" t="n">
+        <v>6323</v>
+      </c>
       <c r="AT40" s="4" t="n"/>
       <c r="AU40" s="4" t="n"/>
       <c r="AV40" s="4" t="n"/>
@@ -17245,7 +17328,9 @@
       <c r="AR41" s="6" t="n">
         <v>12178</v>
       </c>
-      <c r="AS41" s="4" t="n"/>
+      <c r="AS41" s="6" t="n">
+        <v>12922</v>
+      </c>
       <c r="AT41" s="4" t="n"/>
       <c r="AU41" s="4" t="n"/>
       <c r="AV41" s="4" t="n"/>
@@ -17503,7 +17588,9 @@
       <c r="AR42" s="6" t="n">
         <v>475</v>
       </c>
-      <c r="AS42" s="4" t="n"/>
+      <c r="AS42" s="6" t="n">
+        <v>650</v>
+      </c>
       <c r="AT42" s="4" t="n"/>
       <c r="AU42" s="4" t="n"/>
       <c r="AV42" s="4" t="n"/>
@@ -17761,7 +17848,9 @@
       <c r="AR43" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS43" s="4" t="n"/>
+      <c r="AS43" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AT43" s="4" t="n"/>
       <c r="AU43" s="4" t="n"/>
       <c r="AV43" s="4" t="n"/>
@@ -18019,7 +18108,9 @@
       <c r="AR44" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AS44" s="4" t="n"/>
+      <c r="AS44" s="6" t="n">
+        <v>267</v>
+      </c>
       <c r="AT44" s="4" t="n"/>
       <c r="AU44" s="4" t="n"/>
       <c r="AV44" s="4" t="n"/>
@@ -18303,7 +18394,9 @@
       <c r="AR45" s="6" t="n">
         <v>16298</v>
       </c>
-      <c r="AS45" s="4" t="n"/>
+      <c r="AS45" s="6" t="n">
+        <v>16913</v>
+      </c>
       <c r="AT45" s="4" t="n"/>
       <c r="AU45" s="4" t="n"/>
       <c r="AV45" s="4" t="n"/>
@@ -18561,7 +18654,9 @@
       <c r="AR46" s="6" t="n">
         <v>3081</v>
       </c>
-      <c r="AS46" s="4" t="n"/>
+      <c r="AS46" s="6" t="n">
+        <v>3231</v>
+      </c>
       <c r="AT46" s="4" t="n"/>
       <c r="AU46" s="4" t="n"/>
       <c r="AV46" s="4" t="n"/>
@@ -18819,7 +18914,9 @@
       <c r="AR47" s="6" t="n">
         <v>4390</v>
       </c>
-      <c r="AS47" s="4" t="n"/>
+      <c r="AS47" s="6" t="n">
+        <v>4524</v>
+      </c>
       <c r="AT47" s="4" t="n"/>
       <c r="AU47" s="4" t="n"/>
       <c r="AV47" s="4" t="n"/>
@@ -19077,7 +19174,9 @@
       <c r="AR48" s="6" t="n">
         <v>4710</v>
       </c>
-      <c r="AS48" s="4" t="n"/>
+      <c r="AS48" s="6" t="n">
+        <v>5207</v>
+      </c>
       <c r="AT48" s="4" t="n"/>
       <c r="AU48" s="4" t="n"/>
       <c r="AV48" s="4" t="n"/>
@@ -19361,7 +19460,9 @@
       <c r="AR49" s="6" t="n">
         <v>13460</v>
       </c>
-      <c r="AS49" s="4" t="n"/>
+      <c r="AS49" s="6" t="n">
+        <v>13911</v>
+      </c>
       <c r="AT49" s="4" t="n"/>
       <c r="AU49" s="4" t="n"/>
       <c r="AV49" s="4" t="n"/>

</xml_diff>

<commit_message>
Update W2643 ACT snapshot (automatic)
</commit_message>
<xml_diff>
--- a/ACT table.xlsx
+++ b/ACT table.xlsx
@@ -6956,6 +6956,11 @@
           <t>W2642</t>
         </is>
       </c>
+      <c r="AT1" s="0" t="inlineStr">
+        <is>
+          <t>W2643</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="0" t="n">
@@ -7087,7 +7092,9 @@
       <c r="AS2" s="6" t="n">
         <v>7626</v>
       </c>
-      <c r="AT2" s="4" t="n"/>
+      <c r="AT2" s="6" t="n">
+        <v>8004</v>
+      </c>
       <c r="AU2" s="4" t="n"/>
       <c r="AV2" s="4" t="n"/>
       <c r="AW2" s="4" t="n"/>
@@ -7347,7 +7354,9 @@
       <c r="AS3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT3" s="4" t="n"/>
+      <c r="AT3" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU3" s="4" t="n"/>
       <c r="AV3" s="4" t="n"/>
       <c r="AW3" s="4" t="n"/>
@@ -7627,7 +7636,9 @@
       <c r="AS4" s="6" t="n">
         <v>9261</v>
       </c>
-      <c r="AT4" s="4" t="n"/>
+      <c r="AT4" s="6" t="n">
+        <v>9409</v>
+      </c>
       <c r="AU4" s="4" t="n"/>
       <c r="AV4" s="4" t="n"/>
       <c r="AW4" s="4" t="n"/>
@@ -7895,7 +7906,9 @@
       <c r="AS5" s="6" t="n">
         <v>4835</v>
       </c>
-      <c r="AT5" s="4" t="n"/>
+      <c r="AT5" s="6" t="n">
+        <v>4933</v>
+      </c>
       <c r="AU5" s="4" t="n"/>
       <c r="AV5" s="4" t="n"/>
       <c r="AW5" s="4" t="n"/>
@@ -8137,7 +8150,9 @@
       <c r="AS6" s="6" t="n">
         <v>3913</v>
       </c>
-      <c r="AT6" s="4" t="n"/>
+      <c r="AT6" s="6" t="n">
+        <v>5311</v>
+      </c>
       <c r="AU6" s="4" t="n"/>
       <c r="AV6" s="4" t="n"/>
       <c r="AW6" s="4" t="n"/>
@@ -8397,7 +8412,9 @@
       <c r="AS7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT7" s="4" t="n"/>
+      <c r="AT7" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU7" s="4" t="n"/>
       <c r="AV7" s="4" t="n"/>
       <c r="AW7" s="4" t="n"/>
@@ -8657,7 +8674,9 @@
       <c r="AS8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT8" s="4" t="n"/>
+      <c r="AT8" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU8" s="4" t="n"/>
       <c r="AV8" s="4" t="n"/>
       <c r="AW8" s="4" t="n"/>
@@ -8917,7 +8936,9 @@
       <c r="AS9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT9" s="4" t="n"/>
+      <c r="AT9" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU9" s="4" t="n"/>
       <c r="AV9" s="4" t="n"/>
       <c r="AW9" s="4" t="n"/>
@@ -9177,7 +9198,9 @@
       <c r="AS10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT10" s="4" t="n"/>
+      <c r="AT10" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU10" s="4" t="n"/>
       <c r="AV10" s="4" t="n"/>
       <c r="AW10" s="4" t="n"/>
@@ -9437,7 +9460,9 @@
       <c r="AS11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT11" s="4" t="n"/>
+      <c r="AT11" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU11" s="4" t="n"/>
       <c r="AV11" s="4" t="n"/>
       <c r="AW11" s="4" t="n"/>
@@ -9697,7 +9722,9 @@
       <c r="AS12" s="6" t="n">
         <v>21823</v>
       </c>
-      <c r="AT12" s="4" t="n"/>
+      <c r="AT12" s="6" t="n">
+        <v>22626</v>
+      </c>
       <c r="AU12" s="4" t="n"/>
       <c r="AV12" s="4" t="n"/>
       <c r="AW12" s="4" t="n"/>
@@ -9957,7 +9984,9 @@
       <c r="AS13" s="6" t="n">
         <v>162837</v>
       </c>
-      <c r="AT13" s="4" t="n"/>
+      <c r="AT13" s="6" t="n">
+        <v>167108</v>
+      </c>
       <c r="AU13" s="4" t="n"/>
       <c r="AV13" s="4" t="n"/>
       <c r="AW13" s="4" t="n"/>
@@ -10217,7 +10246,9 @@
       <c r="AS14" s="6" t="n">
         <v>26198</v>
       </c>
-      <c r="AT14" s="4" t="n"/>
+      <c r="AT14" s="6" t="n">
+        <v>26971</v>
+      </c>
       <c r="AU14" s="4" t="n"/>
       <c r="AV14" s="4" t="n"/>
       <c r="AW14" s="4" t="n"/>
@@ -10477,7 +10508,9 @@
       <c r="AS15" s="6" t="n">
         <v>1156</v>
       </c>
-      <c r="AT15" s="4" t="n"/>
+      <c r="AT15" s="6" t="n">
+        <v>1444</v>
+      </c>
       <c r="AU15" s="4" t="n"/>
       <c r="AV15" s="4" t="n"/>
       <c r="AW15" s="4" t="n"/>
@@ -10737,7 +10770,9 @@
       <c r="AS16" s="6" t="n">
         <v>2491</v>
       </c>
-      <c r="AT16" s="4" t="n"/>
+      <c r="AT16" s="6" t="n">
+        <v>2632</v>
+      </c>
       <c r="AU16" s="4" t="n"/>
       <c r="AV16" s="4" t="n"/>
       <c r="AW16" s="4" t="n"/>
@@ -10995,7 +11030,9 @@
       <c r="AS17" s="6" t="n">
         <v>1717</v>
       </c>
-      <c r="AT17" s="4" t="n"/>
+      <c r="AT17" s="6" t="n">
+        <v>1717</v>
+      </c>
       <c r="AU17" s="4" t="n"/>
       <c r="AV17" s="4" t="n"/>
       <c r="AW17" s="4" t="n"/>
@@ -11255,7 +11292,9 @@
       <c r="AS18" s="6" t="n">
         <v>1922</v>
       </c>
-      <c r="AT18" s="4" t="n"/>
+      <c r="AT18" s="6" t="n">
+        <v>2025</v>
+      </c>
       <c r="AU18" s="4" t="n"/>
       <c r="AV18" s="4" t="n"/>
       <c r="AW18" s="4" t="n"/>
@@ -11515,7 +11554,9 @@
       <c r="AS19" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT19" s="4" t="n"/>
+      <c r="AT19" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU19" s="4" t="n"/>
       <c r="AV19" s="4" t="n"/>
       <c r="AW19" s="4" t="n"/>
@@ -11775,7 +11816,9 @@
       <c r="AS20" s="6" t="n">
         <v>252</v>
       </c>
-      <c r="AT20" s="4" t="n"/>
+      <c r="AT20" s="6" t="n">
+        <v>331</v>
+      </c>
       <c r="AU20" s="4" t="n"/>
       <c r="AV20" s="4" t="n"/>
       <c r="AW20" s="4" t="n"/>
@@ -12035,7 +12078,9 @@
       <c r="AS21" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT21" s="4" t="n"/>
+      <c r="AT21" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU21" s="4" t="n"/>
       <c r="AV21" s="4" t="n"/>
       <c r="AW21" s="4" t="n"/>
@@ -12295,7 +12340,9 @@
       <c r="AS22" s="6" t="n">
         <v>956</v>
       </c>
-      <c r="AT22" s="4" t="n"/>
+      <c r="AT22" s="6" t="n">
+        <v>992</v>
+      </c>
       <c r="AU22" s="4" t="n"/>
       <c r="AV22" s="4" t="n"/>
       <c r="AW22" s="4" t="n"/>
@@ -12555,7 +12602,9 @@
       <c r="AS23" s="6" t="n">
         <v>1515</v>
       </c>
-      <c r="AT23" s="4" t="n"/>
+      <c r="AT23" s="6" t="n">
+        <v>1515</v>
+      </c>
       <c r="AU23" s="4" t="n"/>
       <c r="AV23" s="4" t="n"/>
       <c r="AW23" s="4" t="n"/>
@@ -12815,7 +12864,9 @@
       <c r="AS24" s="6" t="n">
         <v>3363</v>
       </c>
-      <c r="AT24" s="4" t="n"/>
+      <c r="AT24" s="6" t="n">
+        <v>3506</v>
+      </c>
       <c r="AU24" s="4" t="n"/>
       <c r="AV24" s="4" t="n"/>
       <c r="AW24" s="4" t="n"/>
@@ -13075,7 +13126,9 @@
       <c r="AS25" s="6" t="n">
         <v>877</v>
       </c>
-      <c r="AT25" s="4" t="n"/>
+      <c r="AT25" s="6" t="n">
+        <v>946</v>
+      </c>
       <c r="AU25" s="4" t="n"/>
       <c r="AV25" s="4" t="n"/>
       <c r="AW25" s="4" t="n"/>
@@ -13335,7 +13388,9 @@
       <c r="AS26" s="6" t="n">
         <v>2300</v>
       </c>
-      <c r="AT26" s="4" t="n"/>
+      <c r="AT26" s="6" t="n">
+        <v>2437</v>
+      </c>
       <c r="AU26" s="4" t="n"/>
       <c r="AV26" s="4" t="n"/>
       <c r="AW26" s="4" t="n"/>
@@ -13595,7 +13650,9 @@
       <c r="AS27" s="6" t="n">
         <v>3458</v>
       </c>
-      <c r="AT27" s="4" t="n"/>
+      <c r="AT27" s="6" t="n">
+        <v>3666</v>
+      </c>
       <c r="AU27" s="4" t="n"/>
       <c r="AV27" s="4" t="n"/>
       <c r="AW27" s="4" t="n"/>
@@ -13855,7 +13912,9 @@
       <c r="AS28" s="6" t="n">
         <v>1113</v>
       </c>
-      <c r="AT28" s="4" t="n"/>
+      <c r="AT28" s="6" t="n">
+        <v>1162</v>
+      </c>
       <c r="AU28" s="4" t="n"/>
       <c r="AV28" s="4" t="n"/>
       <c r="AW28" s="4" t="n"/>
@@ -14115,7 +14174,9 @@
       <c r="AS29" s="6" t="n">
         <v>2417</v>
       </c>
-      <c r="AT29" s="4" t="n"/>
+      <c r="AT29" s="6" t="n">
+        <v>2489</v>
+      </c>
       <c r="AU29" s="4" t="n"/>
       <c r="AV29" s="4" t="n"/>
       <c r="AW29" s="4" t="n"/>
@@ -14387,7 +14448,9 @@
       <c r="AS30" s="6" t="n">
         <v>2868</v>
       </c>
-      <c r="AT30" s="4" t="n"/>
+      <c r="AT30" s="6" t="n">
+        <v>2868</v>
+      </c>
       <c r="AU30" s="4" t="n"/>
       <c r="AV30" s="4" t="n"/>
       <c r="AW30" s="4" t="n"/>
@@ -14647,7 +14710,9 @@
       <c r="AS31" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT31" s="4" t="n"/>
+      <c r="AT31" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU31" s="4" t="n"/>
       <c r="AV31" s="4" t="n"/>
       <c r="AW31" s="4" t="n"/>
@@ -14907,7 +14972,9 @@
       <c r="AS32" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT32" s="4" t="n"/>
+      <c r="AT32" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU32" s="4" t="n"/>
       <c r="AV32" s="4" t="n"/>
       <c r="AW32" s="4" t="n"/>
@@ -15167,7 +15234,9 @@
       <c r="AS33" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT33" s="4" t="n"/>
+      <c r="AT33" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU33" s="4" t="n"/>
       <c r="AV33" s="4" t="n"/>
       <c r="AW33" s="4" t="n"/>
@@ -15427,7 +15496,9 @@
       <c r="AS34" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT34" s="4" t="n"/>
+      <c r="AT34" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU34" s="4" t="n"/>
       <c r="AV34" s="4" t="n"/>
       <c r="AW34" s="4" t="n"/>
@@ -15713,7 +15784,9 @@
       <c r="AS35" s="6" t="n">
         <v>8823</v>
       </c>
-      <c r="AT35" s="4" t="n"/>
+      <c r="AT35" s="6" t="n">
+        <v>9030</v>
+      </c>
       <c r="AU35" s="4" t="n"/>
       <c r="AV35" s="4" t="n"/>
       <c r="AW35" s="4" t="n"/>
@@ -15973,7 +16046,9 @@
       <c r="AS36" s="6" t="n">
         <v>1189</v>
       </c>
-      <c r="AT36" s="4" t="n"/>
+      <c r="AT36" s="6" t="n">
+        <v>1244</v>
+      </c>
       <c r="AU36" s="4" t="n"/>
       <c r="AV36" s="4" t="n"/>
       <c r="AW36" s="4" t="n"/>
@@ -16233,7 +16308,9 @@
       <c r="AS37" s="6" t="n">
         <v>1962</v>
       </c>
-      <c r="AT37" s="4" t="n"/>
+      <c r="AT37" s="6" t="n">
+        <v>2170</v>
+      </c>
       <c r="AU37" s="4" t="n"/>
       <c r="AV37" s="4" t="n"/>
       <c r="AW37" s="4" t="n"/>
@@ -16495,7 +16572,9 @@
       <c r="AS38" s="6" t="n">
         <v>6853</v>
       </c>
-      <c r="AT38" s="4" t="n"/>
+      <c r="AT38" s="6" t="n">
+        <v>7283</v>
+      </c>
       <c r="AU38" s="4" t="n"/>
       <c r="AV38" s="4" t="n"/>
       <c r="AW38" s="4" t="n"/>
@@ -16781,7 +16860,9 @@
       <c r="AS39" s="6" t="n">
         <v>14183</v>
       </c>
-      <c r="AT39" s="4" t="n"/>
+      <c r="AT39" s="6" t="n">
+        <v>14770</v>
+      </c>
       <c r="AU39" s="4" t="n"/>
       <c r="AV39" s="4" t="n"/>
       <c r="AW39" s="4" t="n"/>
@@ -17067,7 +17148,9 @@
       <c r="AS40" s="6" t="n">
         <v>6323</v>
       </c>
-      <c r="AT40" s="4" t="n"/>
+      <c r="AT40" s="6" t="n">
+        <v>6555</v>
+      </c>
       <c r="AU40" s="4" t="n"/>
       <c r="AV40" s="4" t="n"/>
       <c r="AW40" s="4" t="n"/>
@@ -17331,7 +17414,9 @@
       <c r="AS41" s="6" t="n">
         <v>12922</v>
       </c>
-      <c r="AT41" s="4" t="n"/>
+      <c r="AT41" s="6" t="n">
+        <v>13541</v>
+      </c>
       <c r="AU41" s="4" t="n"/>
       <c r="AV41" s="4" t="n"/>
       <c r="AW41" s="4" t="n"/>
@@ -17591,7 +17676,9 @@
       <c r="AS42" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="AT42" s="4" t="n"/>
+      <c r="AT42" s="6" t="n">
+        <v>650</v>
+      </c>
       <c r="AU42" s="4" t="n"/>
       <c r="AV42" s="4" t="n"/>
       <c r="AW42" s="4" t="n"/>
@@ -17851,7 +17938,9 @@
       <c r="AS43" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AT43" s="4" t="n"/>
+      <c r="AT43" s="6" t="n">
+        <v>0</v>
+      </c>
       <c r="AU43" s="4" t="n"/>
       <c r="AV43" s="4" t="n"/>
       <c r="AW43" s="4" t="n"/>
@@ -18111,7 +18200,9 @@
       <c r="AS44" s="6" t="n">
         <v>267</v>
       </c>
-      <c r="AT44" s="4" t="n"/>
+      <c r="AT44" s="6" t="n">
+        <v>306</v>
+      </c>
       <c r="AU44" s="4" t="n"/>
       <c r="AV44" s="4" t="n"/>
       <c r="AW44" s="4" t="n"/>
@@ -18397,7 +18488,9 @@
       <c r="AS45" s="6" t="n">
         <v>16913</v>
       </c>
-      <c r="AT45" s="4" t="n"/>
+      <c r="AT45" s="6" t="n">
+        <v>17487</v>
+      </c>
       <c r="AU45" s="4" t="n"/>
       <c r="AV45" s="4" t="n"/>
       <c r="AW45" s="4" t="n"/>
@@ -18657,7 +18750,9 @@
       <c r="AS46" s="6" t="n">
         <v>3231</v>
       </c>
-      <c r="AT46" s="4" t="n"/>
+      <c r="AT46" s="6" t="n">
+        <v>3380</v>
+      </c>
       <c r="AU46" s="4" t="n"/>
       <c r="AV46" s="4" t="n"/>
       <c r="AW46" s="4" t="n"/>
@@ -18917,7 +19012,9 @@
       <c r="AS47" s="6" t="n">
         <v>4524</v>
       </c>
-      <c r="AT47" s="4" t="n"/>
+      <c r="AT47" s="6" t="n">
+        <v>4660</v>
+      </c>
       <c r="AU47" s="4" t="n"/>
       <c r="AV47" s="4" t="n"/>
       <c r="AW47" s="4" t="n"/>
@@ -19177,7 +19274,9 @@
       <c r="AS48" s="6" t="n">
         <v>5207</v>
       </c>
-      <c r="AT48" s="4" t="n"/>
+      <c r="AT48" s="6" t="n">
+        <v>5207</v>
+      </c>
       <c r="AU48" s="4" t="n"/>
       <c r="AV48" s="4" t="n"/>
       <c r="AW48" s="4" t="n"/>
@@ -19463,7 +19562,9 @@
       <c r="AS49" s="6" t="n">
         <v>13911</v>
       </c>
-      <c r="AT49" s="4" t="n"/>
+      <c r="AT49" s="6" t="n">
+        <v>14546</v>
+      </c>
       <c r="AU49" s="4" t="n"/>
       <c r="AV49" s="4" t="n"/>
       <c r="AW49" s="4" t="n"/>

</xml_diff>